<commit_message>
feat: npm run add-game 스크립트 추가 (게임추가+매칭+빌드 one-shot)
npm run add-game 게임명 → 5단계 자동 실행

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/game-system/game-data/library/2-ledger/cottage-owned-games-ledger.xlsx
+++ b/game-system/game-data/library/2-ledger/cottage-owned-games-ledger.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4141" uniqueCount="1351">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4145" uniqueCount="1352">
   <si>
     <t xml:space="preserve"> &lt;필터 바꾸셔도 됩니다&gt;</t>
   </si>
@@ -3991,6 +3991,9 @@
   </si>
   <si>
     <t>인코딩테스트</t>
+  </si>
+  <si>
+    <t>에이다의꿈</t>
   </si>
   <si>
     <t>보유게임리스트는 탭을 이동해주세요</t>
@@ -5344,7 +5347,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AB1048"/>
+  <dimension ref="A1:AB1049"/>
   <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="12.63" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16.38" customWidth="1"/>
@@ -33851,6 +33854,23 @@
         <v>1311</v>
       </c>
       <c r="E1048">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1049" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1049" t="s">
+        <v>1314</v>
+      </c>
+      <c r="B1049" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1049" t="s">
+        <v>1311</v>
+      </c>
+      <c r="D1049" t="s">
+        <v>1311</v>
+      </c>
+      <c r="E1049">
         <v>0</v>
       </c>
     </row>
@@ -34026,7 +34046,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="93" t="s">
-        <v>1314</v>
+        <v>1315</v>
       </c>
       <c r="B1" s="47"/>
     </row>
@@ -34036,10 +34056,10 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="47" t="s">
-        <v>1315</v>
+        <v>1316</v>
       </c>
       <c r="B3" s="47" t="s">
-        <v>1316</v>
+        <v>1317</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -34056,10 +34076,10 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="47" t="s">
-        <v>1317</v>
+        <v>1318</v>
       </c>
       <c r="B6" s="47" t="s">
-        <v>1318</v>
+        <v>1319</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -34070,18 +34090,18 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="47" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
       <c r="B8" s="47" t="s">
-        <v>1320</v>
+        <v>1321</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="47" t="s">
-        <v>1321</v>
+        <v>1322</v>
       </c>
       <c r="B9" s="47" t="s">
-        <v>1322</v>
+        <v>1323</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -34098,10 +34118,10 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="47" t="s">
-        <v>1323</v>
+        <v>1324</v>
       </c>
       <c r="B12" s="47" t="s">
-        <v>1324</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -34118,10 +34138,10 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="47" t="s">
-        <v>1325</v>
+        <v>1326</v>
       </c>
       <c r="B15" s="47" t="s">
-        <v>1326</v>
+        <v>1327</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -34181,7 +34201,7 @@
     </row>
     <row r="27" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B27" s="47" t="s">
-        <v>1327</v>
+        <v>1328</v>
       </c>
     </row>
   </sheetData>
@@ -34198,7 +34218,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="93" t="s">
-        <v>1314</v>
+        <v>1315</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -34206,126 +34226,126 @@
     </row>
     <row r="3" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B3" s="47" t="s">
-        <v>1328</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="47" t="s">
-        <v>1329</v>
+        <v>1330</v>
       </c>
       <c r="B4" s="47"/>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="47" t="s">
-        <v>1330</v>
+        <v>1331</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="47" t="s">
-        <v>1331</v>
+        <v>1332</v>
       </c>
       <c r="B6" s="47"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="47" t="s">
-        <v>1332</v>
+        <v>1333</v>
       </c>
       <c r="B7" s="47"/>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="47" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
       <c r="B8" s="47"/>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="47" t="s">
-        <v>1334</v>
+        <v>1335</v>
       </c>
       <c r="B9" s="47"/>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="47" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="B10" s="47" t="s">
-        <v>1336</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="47" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B11" s="47"/>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="47" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="47" t="s">
-        <v>1339</v>
+        <v>1340</v>
       </c>
       <c r="B13" s="47"/>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="47" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="47" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="B15" s="47"/>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" s="47" t="s">
-        <v>1342</v>
+        <v>1343</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="47" t="s">
-        <v>1343</v>
+        <v>1344</v>
       </c>
       <c r="B17" s="47"/>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="47" t="s">
-        <v>1344</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="47" t="s">
-        <v>1345</v>
+        <v>1346</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="47" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="B20" s="47"/>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="47" t="s">
-        <v>1347</v>
+        <v>1348</v>
       </c>
       <c r="B21" s="47"/>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="47" t="s">
-        <v>1348</v>
+        <v>1349</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="47" t="s">
-        <v>1349</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="47" t="s">
-        <v>1350</v>
+        <v>1351</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: add-owned-game.js 소스 xlsx 참조 버그 수정 + 신규 게임 5종 추가
- add-owned-game: ledger xlsx → source xlsx로 수정 (build-master 연동)
- 신규 추가: 원드러스크리처, 천국과맥주, 글렌모어연대기, 딥씨크루, 에이다의꿈
- 총 게임 수: 636 → 641

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/game-system/game-data/library/2-ledger/cottage-owned-games-ledger.xlsx
+++ b/game-system/game-data/library/2-ledger/cottage-owned-games-ledger.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4145" uniqueCount="1352">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4161" uniqueCount="1356">
   <si>
     <t xml:space="preserve"> &lt;필터 바꾸셔도 됩니다&gt;</t>
   </si>
@@ -3994,6 +3994,18 @@
   </si>
   <si>
     <t>에이다의꿈</t>
+  </si>
+  <si>
+    <t>원드러스크리처</t>
+  </si>
+  <si>
+    <t>천국과맥주</t>
+  </si>
+  <si>
+    <t>글렌모어연대기</t>
+  </si>
+  <si>
+    <t>딥씨크루</t>
   </si>
   <si>
     <t>보유게임리스트는 탭을 이동해주세요</t>
@@ -5347,7 +5359,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AB1049"/>
+  <dimension ref="A1:AB1053"/>
   <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="12.63" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16.38" customWidth="1"/>
@@ -33871,6 +33883,74 @@
         <v>1311</v>
       </c>
       <c r="E1049">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1050" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1050" t="s">
+        <v>1315</v>
+      </c>
+      <c r="B1050" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1050" t="s">
+        <v>1311</v>
+      </c>
+      <c r="D1050" t="s">
+        <v>1311</v>
+      </c>
+      <c r="E1050">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1051" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1051" t="s">
+        <v>1316</v>
+      </c>
+      <c r="B1051" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1051" t="s">
+        <v>1311</v>
+      </c>
+      <c r="D1051" t="s">
+        <v>1311</v>
+      </c>
+      <c r="E1051">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1052" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1052" t="s">
+        <v>1317</v>
+      </c>
+      <c r="B1052" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1052" t="s">
+        <v>1311</v>
+      </c>
+      <c r="D1052" t="s">
+        <v>1311</v>
+      </c>
+      <c r="E1052">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1053" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1053" t="s">
+        <v>1318</v>
+      </c>
+      <c r="B1053" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1053" t="s">
+        <v>1311</v>
+      </c>
+      <c r="D1053" t="s">
+        <v>1311</v>
+      </c>
+      <c r="E1053">
         <v>0</v>
       </c>
     </row>
@@ -34046,7 +34126,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="93" t="s">
-        <v>1315</v>
+        <v>1319</v>
       </c>
       <c r="B1" s="47"/>
     </row>
@@ -34056,10 +34136,10 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="47" t="s">
-        <v>1316</v>
+        <v>1320</v>
       </c>
       <c r="B3" s="47" t="s">
-        <v>1317</v>
+        <v>1321</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -34076,10 +34156,10 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="47" t="s">
-        <v>1318</v>
+        <v>1322</v>
       </c>
       <c r="B6" s="47" t="s">
-        <v>1319</v>
+        <v>1323</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -34090,18 +34170,18 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="47" t="s">
-        <v>1320</v>
+        <v>1324</v>
       </c>
       <c r="B8" s="47" t="s">
-        <v>1321</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="47" t="s">
-        <v>1322</v>
+        <v>1326</v>
       </c>
       <c r="B9" s="47" t="s">
-        <v>1323</v>
+        <v>1327</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -34118,10 +34198,10 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="47" t="s">
-        <v>1324</v>
+        <v>1328</v>
       </c>
       <c r="B12" s="47" t="s">
-        <v>1325</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -34138,10 +34218,10 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="47" t="s">
-        <v>1326</v>
+        <v>1330</v>
       </c>
       <c r="B15" s="47" t="s">
-        <v>1327</v>
+        <v>1331</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -34201,7 +34281,7 @@
     </row>
     <row r="27" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B27" s="47" t="s">
-        <v>1328</v>
+        <v>1332</v>
       </c>
     </row>
   </sheetData>
@@ -34218,7 +34298,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="93" t="s">
-        <v>1315</v>
+        <v>1319</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -34226,126 +34306,126 @@
     </row>
     <row r="3" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B3" s="47" t="s">
-        <v>1329</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="47" t="s">
-        <v>1330</v>
+        <v>1334</v>
       </c>
       <c r="B4" s="47"/>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="47" t="s">
-        <v>1331</v>
+        <v>1335</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="47" t="s">
-        <v>1332</v>
+        <v>1336</v>
       </c>
       <c r="B6" s="47"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="47" t="s">
-        <v>1333</v>
+        <v>1337</v>
       </c>
       <c r="B7" s="47"/>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="47" t="s">
-        <v>1334</v>
+        <v>1338</v>
       </c>
       <c r="B8" s="47"/>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="47" t="s">
-        <v>1335</v>
+        <v>1339</v>
       </c>
       <c r="B9" s="47"/>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="47" t="s">
-        <v>1336</v>
+        <v>1340</v>
       </c>
       <c r="B10" s="47" t="s">
-        <v>1337</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="47" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B11" s="47"/>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="47" t="s">
-        <v>1339</v>
+        <v>1343</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="47" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B13" s="47"/>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="47" t="s">
-        <v>1341</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="47" t="s">
-        <v>1342</v>
+        <v>1346</v>
       </c>
       <c r="B15" s="47"/>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" s="47" t="s">
-        <v>1343</v>
+        <v>1347</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="47" t="s">
-        <v>1344</v>
+        <v>1348</v>
       </c>
       <c r="B17" s="47"/>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="47" t="s">
-        <v>1345</v>
+        <v>1349</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="47" t="s">
-        <v>1346</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="47" t="s">
-        <v>1347</v>
+        <v>1351</v>
       </c>
       <c r="B20" s="47"/>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="47" t="s">
-        <v>1348</v>
+        <v>1352</v>
       </c>
       <c r="B21" s="47"/>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="47" t="s">
-        <v>1349</v>
+        <v>1353</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="47" t="s">
-        <v>1350</v>
+        <v>1354</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="47" t="s">
-        <v>1351</v>
+        <v>1355</v>
       </c>
     </row>
   </sheetData>

</xml_diff>